<commit_message>
docs(shotlist): staff-facing Korean Excel and i18n data for 2026-04-27
- xlsx: Korean sheet names and column headers; P0 priority fill; 3시트(샷리스트, 페이지별 요약, 촬영 일정)
- Row copy: 52 lines in Korean (scripts/shotlist_ko_p0|p1|p2, merged to photo-shotlist-ko.json)
- Keep English structural base (photo-shotlist-base-en.json) for dev merge; run merge_shotlist_ko.py to regenerate
- md: same table with Korean column titles + Korean intro
- build-photo-shotlist.py: load KO JSON, fix markdown join bug

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/photo-shotlist-2026-04-27.xlsx
+++ b/docs/photo-shotlist-2026-04-27.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Shotlist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary by Page" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Shoot Day Plan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="샷리스트" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="페이지별 요약" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="촬영 일정" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Shotlist'!$A$1:$Q$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'샷리스트'!$A$1:$Q$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -487,108 +487,108 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="56" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="44" customWidth="1" min="12" max="12"/>
     <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
     <col width="50" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="50" customWidth="1" min="17" max="17"/>
+    <col width="52" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>priority</t>
+          <t>우선순위 (P0=최우선)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>page</t>
+          <t>페이지(URL/범주)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>page_file</t>
+          <t>소스 파일(개발)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>section</t>
+          <t>섹션·촬영 위치</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>current_state</t>
+          <t>현재 웹 상태</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>photo_subject</t>
+          <t>촬영·연출(무엇을 담을지)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>composition</t>
+          <t>구도</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>orientation</t>
+          <t>화면 비율</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>min_resolution</t>
+          <t>최소 해상도</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>mood_lighting</t>
+          <t>조명·무드</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>must_include</t>
+          <t>반드시 포함</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>must_avoid</t>
+          <t>절대 피할 것</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>consent_required</t>
+          <t>초상·동의</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>suggested_filename</t>
+          <t>제안 파일 경로(개발)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>촬영 장수</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>비고</t>
         </is>
       </c>
     </row>
@@ -615,27 +615,27 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Hero (poster fallback for /hero-video.mp4)</t>
+          <t>메인 히어로(동영상·포스터 대체용, /hero-video.mp4)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>video w/ /main.jpeg poster</t>
+          <t>동영상 + /main.jpeg 포스터</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Wide cinematic shot of Tune Clinic Apgujeong building exterior at golden hour with subtle gold accent lighting; signage legible. Used as &lt;video poster&gt; when video fails or is suppressed.</t>
+          <t>골든아워의 압구정 병원 외부 와이드. 골드 포인트 조명, 간판 식별 용이. 동영상 미로딩·억제 시 &lt;video poster&gt;로 사용.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -645,22 +645,22 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>warm golden hour, premium</t>
+          <t>따뜻한 골든아워, 프리미엄 톤</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>Tune Clinic signage, 5th-floor building facade, clean storefront</t>
+          <t>튠의원(또는 클리닉) 식별 간판, 5층 전면, 깔끔한 상가 외관</t>
         </is>
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>passersby faces, license plates, competing clinic signs in same frame</t>
+          <t>행인 얼굴, 자동차 번호판, 동일 화면에 경쟁 클리닉 식별 간판</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -670,12 +670,12 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>3 angles, 1 final</t>
+          <t>각도 3장 + 최종 1장</t>
         </is>
       </c>
       <c r="Q2" s="4" t="inlineStr">
         <is>
-          <t>Also produce a square 1:1 crop for OG; align horizon with rule-of-thirds so headline overlay (left-bottom) stays uncluttered.</t>
+          <t>OG용 1:1 정사각 크롭도. 수평선 3분할, 좌하단에 헤드라인·텍스트 오버레이 여백.</t>
         </is>
       </c>
     </row>
@@ -702,27 +702,27 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Hero (alternate interior poster)</t>
+          <t>메인 히어로(실내 대체 포스터)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>video w/ /main.jpeg poster</t>
+          <t>동영상 + /main.jpeg 포스터</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Signature interior wide of consultation room or main hallway with gold accent + warm wood — composed dark on edges so white serif headline reads.</t>
+          <t>상담실 또는 메인 복도 시그니처 실내. 골드 포인트·웜우드, 가장자리는 어둡게(화이트 타이틀 가독).</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -732,22 +732,22 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>soft moody premium, warm tungsten</t>
+          <t>은은한 뮤지엄톤, 따뜻한 텅스텐</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>clinic interior detail (gold trim, wood, plants), uncluttered surface</t>
+          <t>실내 골드 테두리·우드·식물, 정돈된 면</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>staff faces (unless released), patient personal items, glare on glass</t>
+          <t>얼굴(동의 없을 때), 환자 소지품, 유리 눈부심</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -757,12 +757,12 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2 angles</t>
+          <t>각도 2장</t>
         </is>
       </c>
       <c r="Q3" s="4" t="inlineStr">
         <is>
-          <t>Optional secondary poster; leave 40% negative space on left for headline.</t>
+          <t>보조 포스터. 왼쪽 40% 네거티브 스페이스(헤드라인용).</t>
         </is>
       </c>
     </row>
@@ -789,27 +789,27 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Why Apgujeong (trust strip, line 124)</t>
+          <t>Why Apgujeong(신뢰 스트립, 124행 부근)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Apgujeong-rodeo street view from clinic's 5th-floor window OR from sidewalk looking up at building — establishes the district context.</t>
+          <t>5층 창가에서의 압구정 로데 거리, 또는 보도에서 건물을 올려다보는 뷰(지구 맥락).</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -819,22 +819,22 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>bright daylight, slightly desaturated premium</t>
+          <t>밝은 주광, 살짝 낮은 채도(프리미엄 느낌)</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>recognizable Apgujeong streetscape (boutiques, tree-lined road)</t>
+          <t>압구정 거리(부티크·가로수) 식별 가능</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>identifiable pedestrians, brand logos of luxury houses without permission</t>
+          <t>얼굴 식별되는 행인, 허락 없는 명품 악센트 로고</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -844,12 +844,12 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2장</t>
         </is>
       </c>
       <c r="Q4" s="4" t="inlineStr">
         <is>
-          <t>Reuses on /apgujeong-aesthetic-clinic-for-foreign-patients.html and /international-patients-guide.html.</t>
+          <t>외국인 환자 가이드·압구정 페이지에 재사용.</t>
         </is>
       </c>
     </row>
@@ -876,27 +876,27 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Inside the Clinic (line 1256, dark CTA section)</t>
+          <t>Inside the Clinic(다크 CTA, 1256행)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Reception desk with concierge member greeting (back-of-head only or signed-release talent), warm lamp, gold accent visible.</t>
+          <t>리셉션 데스크, 컨시어지(뒷머리만 또는 합의된 인물), 램프, 골드 악센트.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -906,22 +906,22 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>warm tungsten, evening premium</t>
+          <t>따뜻한 텅스텐, 이브닝 느낌</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>reception counter, branded signage subtle, fresh florals</t>
+          <t>카운터, 은은한 브랜드, 생화</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>visible patient face, prices on monitor, paperwork with names</t>
+          <t>환자 얼굴, 모니터 가격, 이름 적힌 서류</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Yes (staff release)</t>
+          <t>필요(직원·초상)</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -931,12 +931,12 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>3 angles</t>
+          <t>각도 3장</t>
         </is>
       </c>
       <c r="Q5" s="4" t="inlineStr">
         <is>
-          <t>This block is currently 100% text on dark; image is high-impact.</t>
+          <t>현재 100% 텍스트 — 이미지 투입 시 임팩트 큼.</t>
         </is>
       </c>
     </row>
@@ -963,27 +963,27 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Visit Us (line 1335 - location/map block)</t>
+          <t>Visit Us(지도·주소 블록, 1335행)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>5th-floor elevator landing or floor signage immediately outside clinic door — orientation cue for arriving patients.</t>
+          <t>5층 엘리베이터홀·클리닉 문 바로 앞 층수 안내(방문 동선).</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -993,22 +993,22 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral</t>
+          <t>밝은 클리니컬</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>floor number visible, clinic logo on door/wall, polished floor</t>
+          <t>층수 표기, 벽/문에 로고, 광택 바닥</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>other tenants' signage in same frame, cleaning carts</t>
+          <t>다른 임대인 간판, 청소 카트</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -1018,12 +1018,12 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2장</t>
         </is>
       </c>
       <c r="Q6" s="4" t="inlineStr">
         <is>
-          <t>Pairs naturally next to the address text + map embed.</t>
+          <t>주소+지도 옆에 배치.</t>
         </is>
       </c>
     </row>
@@ -1050,27 +1050,27 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 4)</t>
+          <t>예약 Hero(4행)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>text only, gold underline only</t>
+          <t>텍스트·골드 밑줄만</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Calm consultation desk overhead — leather notebook, clinic-branded card, fountain pen, single fresh stem in vase, soft hands of physician (Dr. Cha or Dr. Ju) writing a plan.</t>
+          <t>탑뷰: 가죽 다이어리, 클리닉 명함, 만년필, 꽃 한 송이, (차/주 원장) 손이 플랜을 작성.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -1080,22 +1080,22 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>soft daylight from left, premium calm</t>
+          <t>좌측 데이라이트, 침·차분</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>hand in white-coat cuff, branded card, planning notebook</t>
+          <t>흰 가운 소매, 브랜딩, 플랜 수첩</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>real patient name on card, phone screens with private content</t>
+          <t>진짜 환자 이름, 개인이 보이는 화면</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Yes (physician release)</t>
+          <t>필요(의사)</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -1105,12 +1105,12 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>3 variants</t>
+          <t>변형 3장</t>
         </is>
       </c>
       <c r="Q7" s="4" t="inlineStr">
         <is>
-          <t>Doubles as 'plan with the doctor' visual; reuse across decision-protection and design-method.</t>
+          <t>의사와 함께하는 플랜’ 비주얼, 결정보호·디자인방식 재사용.</t>
         </is>
       </c>
     </row>
@@ -1137,27 +1137,27 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Booking confirmation success state (line 200)</t>
+          <t>예약 완료(성공) 화면(200행)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>text only with green checkmark</t>
+          <t>체크+텍스트</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Soft macro of fresh florals + 'Welcome' note card on reception counter — used as gentle reassurance image after booking.</t>
+          <t>리셉션에 화이트·크림 꽃 + 환영 카드 클로즈(제출 직후 안심).</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>square (1:1)</t>
+          <t>정사각 1:1</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1167,22 +1167,22 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>soft daylight, airy</t>
+          <t>밝고 에어리</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>florals (white/cream), branded card or envelope</t>
+          <t>꽃, 브랜딩 카드/봉투</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>any text that could date the image, patient names</t>
+          <t>시기 티 나는 문구, 환자 이름</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1192,12 +1192,12 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2장</t>
         </is>
       </c>
       <c r="Q8" s="4" t="inlineStr">
         <is>
-          <t>Optional but elevates UX after submit.</t>
+          <t>UX 고급화(선택).</t>
         </is>
       </c>
     </row>
@@ -1224,27 +1224,27 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 35) — flagship LP</t>
+          <t>메타셀 LP Hero(35행, 핵심 랜딩)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>text only on dark gradient</t>
+          <t>다크 그라데이션·텍스트</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Physician hands (gloved) holding a labeled PRP centrifuge tube against a soft bokeh of treatment-room lighting; alternate take with PBM device head in foreground.</t>
+          <t>장갑 낀 손이 라벨된 PRP 원심분리 관을 들거나, PBM 헤드 전경. 시술실 보케.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1254,22 +1254,22 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>soft moody premium, blue-warm split</t>
+          <t>뮤지엄톤, 쿨·웜 스플릿</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>gloved hands, PRP tube OR PBM device, white-coat cuff</t>
+          <t>장갑, PRP 관·또는 PBM, 흰 가운 커프</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>any 'stem cell' wording on labels (regulatory), patient body parts</t>
+          <t>‘줄기세포’ 등 오해 소지 문구(라벨), 환자 신체</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Yes (physician release)</t>
+          <t>필요(의사)</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1279,12 +1279,12 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>4 variants</t>
+          <t>변형 4장</t>
         </is>
       </c>
       <c r="Q9" s="4" t="inlineStr">
         <is>
-          <t>Critical for ad launch. Compose dark-left so white headline reads.</t>
+          <t>광고 런칭 핵심. 좌측 다크(화이트 헤드라인 가독).</t>
         </is>
       </c>
     </row>
@@ -1311,27 +1311,27 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Autologous regenerative explainer (line 80)</t>
+          <t>자가 PRP·재생 설명(80행)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>PRP centrifuge machine on stainless tray with prepared tubes mid-process — clean clinical scene.</t>
+          <t>스텐 트레이 위 원심분리기·준비된 튜브(진행 중) 클리니컬 톤.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1341,22 +1341,22 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral</t>
+          <t>밝은 클리니컬</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>centrifuge, labeled tubes (Tune Clinic label OK), gloved hand entering frame</t>
+          <t>원심분리기, (튠 클리닉 라벨) 튜브, 장갑</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>cluttered countertop, expired-looking labels</t>
+          <t>지저분한 판, 유통기한 지난 라벨</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -1366,12 +1366,12 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>3 angles</t>
+          <t>각도 3장</t>
         </is>
       </c>
       <c r="Q10" s="4" t="inlineStr">
         <is>
-          <t>Equipment close-up reused on collagen-builder + skin-boosters pages.</t>
+          <t>콜라겐·스킨부스터도 재사용.</t>
         </is>
       </c>
     </row>
@@ -1398,27 +1398,27 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Three illustrative builds (line 109)</t>
+          <t>3가지 구성(109행, 카드 그리드)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>text only, three card grid</t>
+          <t>텍스트만(3칸)</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Three matched square crops: (a) Ultherapy device handpiece, (b) Thermage tip on machine, (c) PBM device head — same lighting setup so cards align.</t>
+          <t>동일 조명: (a)울쎄라 핸드피스 (b)써마지 팁+기기 (c)PBM 헤드 — 정사각 셋이 정렬.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>square (1:1)</t>
+          <t>정사각 1:1</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1428,22 +1428,22 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral with single warm rim light</t>
+          <t>클리니컬+웜 림라이트</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>device branding faintly visible, dust-free surfaces</t>
+          <t>은은한 제품 밍, 먼지 없는 면</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>serial numbers, mismatched lighting between the three</t>
+          <t>시리얼, 셋 간 조명 불일치</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1453,12 +1453,12 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>3 (one per build)</t>
+          <t>3장(구성당 1)</t>
         </is>
       </c>
       <c r="Q11" s="4" t="inlineStr">
         <is>
-          <t>Shoot all three back-to-back with same lighting to keep card grid consistent.</t>
+          <t>연속 촬영으로 카드 격자 통일감.</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1485,27 +1485,27 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Dr. Cha — formal portrait</t>
+          <t>차승연 원장 — 정식(반신) 초상(메디컬보드 893행 등)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>initials avatar / text only</t>
+          <t>이니셜/텍스트</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Dr. Seung Yeon Cha, Representative Director — half-body in white coat against warm neutral wall, calm confident expression looking just off-camera.</t>
+          <t>대표·원장, 웜뉴트럴 벽, 자신감·차분, 시선은 카메라 살짝 옆.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>portrait</t>
+          <t>인물(세로)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>portrait (4:5)</t>
+          <t>세로 4:5</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1515,22 +1515,22 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>soft window daylight + bounce, premium clinical</t>
+          <t>소프트 윈도+바운스, 프리미엄 클리닉</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>white coat with subtle Tune branding, name pin if available, neutral background</t>
+          <t>흰 가운·은은한 브랜딩, 네임핀(가능시)</t>
         </is>
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>strong shadows, busy background, distracting jewelry</t>
+          <t>강한 그림자, 산만한 배경, 과한 액세서리</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Yes (physician release)</t>
+          <t>필요(의사)</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>3 variants (head-shot, half-body, full)</t>
+          <t>얼굴·반신·전신 변형 3</t>
         </is>
       </c>
       <c r="Q12" s="4" t="inlineStr">
         <is>
-          <t>Most-used asset on the site. Capture matching landscape crop too (3:2).</t>
+          <t>사이트 전역 최빈도. 3:2 풍경도 동시 촬영.</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1572,27 +1572,27 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Dr. Cha — environmental</t>
+          <t>차승연 원장 — 환경(상담)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Dr. Cha at consultation desk, half-body, looking at patient chart / tablet (no patient face visible) — body angled 30deg from camera.</t>
+          <t>상담 데스크, 환자차트/태블릿(얼굴 X), 30° 각도.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1602,22 +1602,22 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>warm natural daylight from window-left</t>
+          <t>창가 좌측 데이라이트</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>consultation chair, planning notebook, gold accent</t>
+          <t>의자, 수첩, 골드 포인트</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>real patient identifiers on chart, screen content with names</t>
+          <t>차트·화면에 실명, 식별자</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Yes (physician release)</t>
+          <t>필요(의사)</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -1627,12 +1627,12 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3장</t>
         </is>
       </c>
       <c r="Q13" s="4" t="inlineStr">
         <is>
-          <t>Used on /booking, /design-method, /decision-protection, /metacell-protocol footer CTAs.</t>
+          <t>예약·디자인방식·결정보호·메타셀 푸터 CTA</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1659,27 +1659,27 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Dr. Ju — formal portrait</t>
+          <t>주지훈 원장 — 정식(반신) 초상</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>initials avatar / text only</t>
+          <t>이니셜/텍스트</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Dr. Jee Hoon Ju, International Director — half-body in white coat, friendly approachable expression, slight smile, looking at camera.</t>
+          <t>인터내셔널 디렉터, 흰 가운, 친근·열려있는 인상(영어 환자용).</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>portrait</t>
+          <t>인물(세로)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>portrait (4:5)</t>
+          <t>세로 4:5</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1689,22 +1689,22 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>soft window daylight + bounce, premium clinical</t>
+          <t>소프트 윈도+바운스</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>white coat, English-speaking-lead-friendly demeanor, neutral background</t>
+          <t>흰 가운, 국제·친화적 인상</t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>overly serious/clinical mood — should read 'approachable' for international patients</t>
+          <t>과도하게 딱딱/무서움(외국인 이탈)</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Yes (physician release)</t>
+          <t>필요(의사)</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -1714,12 +1714,12 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>3 variants</t>
+          <t>변형 3</t>
         </is>
       </c>
       <c r="Q14" s="4" t="inlineStr">
         <is>
-          <t>Pair with matching landscape crop for use as English-language LP author byline.</t>
+          <t>LP 저자 byline·영어용 가로 crop.</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1746,27 +1746,27 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Dr. Ju — environmental (English consult)</t>
+          <t>주지훈 원장 — 영어 상담(환경)</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Dr. Ju at consultation table with iPad showing planning visual, gesturing in conversation across desk (back-of-head of stand-in patient OK).</t>
+          <t>iPad(플랜), 데스크 건너 대화(스탠드인·뒷통수만), 제스처.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1776,22 +1776,22 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>warm daylight + warm tungsten fill</t>
+          <t>데이+텅스텐 필</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>iPad with planning visual (placeholder), Tune card, two chairs</t>
+          <t>아이패드(플랜), 명함, 의자 2</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>real patient face, real chart data on iPad</t>
+          <t>진짜 환자 얼굴, 식별 데이터</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Yes (physician + stand-in release)</t>
+          <t>필요(의사+스탠드인)</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -1801,12 +1801,12 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3장</t>
         </is>
       </c>
       <c r="Q15" s="4" t="inlineStr">
         <is>
-          <t>Anchors English-speaking concierge story across booking + international guide.</t>
+          <t>영어·컨시어지 스토리, 예약·가이드</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1833,27 +1833,27 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Building exterior wide</t>
+          <t>건물 전면(넓은 화면)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Wide street-level shot of 868 Nonhyeon-ro building, full facade with 5th-floor location identifiable; pedestrian-free if possible.</t>
+          <t>논현로 868 전면(5층 식별), 보행자 적은 앵글.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1863,22 +1863,22 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>bright midday daylight (sunny window 11am)</t>
+          <t>한낮 맑은 날(11시 전후 권장)</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>full building, street-level context, address number subtle</t>
+          <t>전면, 가로·주소 맥락</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>people in the frame, parked cars dominating</t>
+          <t>지배적 행인, 번호판 클로즈</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -1888,12 +1888,12 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>3 (different focal lengths)</t>
+          <t>초점거리 3가지</t>
         </is>
       </c>
       <c r="Q16" s="4" t="inlineStr">
         <is>
-          <t>Reused as OG image candidate for apgujeong page.</t>
+          <t>압구정 페이지 OG 후보.</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1920,27 +1920,27 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>5th-floor reception (location proof)</t>
+          <t>5층 대기/리셥션(위치 증빙)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Reception/waiting lounge wide — clean waiting seats, tea station, branded panel, plant.</t>
+          <t>대기 넓이, 티·플랜트, 벽면 브랜딩(환자 없이).</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1950,22 +1950,22 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>warm daylight + accent lighting</t>
+          <t>따뜻한 데이+액센트</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>branded wall, comfortable seating, tea/water station, fresh flowers</t>
+          <t>브랜딩, 좌석, 티/워터</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>patients in waiting, magazines with names</t>
+          <t>대기 환자, 이름 있는 잡지</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -1975,12 +1975,12 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>3 angles</t>
+          <t>각도 3</t>
         </is>
       </c>
       <c r="Q17" s="4" t="inlineStr">
         <is>
-          <t>Shoot before clinic opens for empty waiting area.</t>
+          <t>오픈 전 공실이면 베스트.</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2007,27 +2007,27 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Apgujeong-rodeo street context</t>
+          <t>압구정·로데 거리 맥락</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Apgujeong-rodeo street scene mid-block — boutique storefronts, tree canopy, leaves, premium district vibe.</t>
+          <t>로데 미드블록 — 부티크, 가로수, 프리미엄가 압구정 무드.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -2037,22 +2037,22 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>bright daylight, slightly desaturated</t>
+          <t>밝고 살짝 desat</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>recognizable Apgujeong-rodeo streetscape</t>
+          <t>압구정 로데 식별</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>identifiable individual pedestrians, competitor clinics</t>
+          <t>얼굴 식별, 경쟁 클리닉</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -2062,12 +2062,12 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>4 (variations)</t>
+          <t>4 변형</t>
         </is>
       </c>
       <c r="Q18" s="4" t="inlineStr">
         <is>
-          <t>Multi-page reuse — home, apgujeong page, international guide, blog hero pool.</t>
+          <t>홈·가이드·블로그 풀 재사용.</t>
         </is>
       </c>
     </row>
@@ -2094,27 +2094,27 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 37)</t>
+          <t>시그니처 리프팅 LP Hero(37행)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>text only on dark</t>
+          <t>다크 배경·텍스트</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Ultherapy device with handpiece in physician's hand, mid-treatment angle (no patient face) — handpiece resting on neutral pad with gel.</t>
+          <t>울쎄라+핸드피스, 의사 손(얼굴X), 젤+패드 위(중간 촬영 앵글).</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -2124,22 +2124,22 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>soft moody premium, dark backdrop</t>
+          <t>뮤지엄톤, 다크 백</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Ultherapy branding visible but subtle, gloved hand</t>
+          <t>울쎄라 밍, 장갑</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>patient face, procedure-in-progress with skin visible</t>
+          <t>환자 얼·피부 노출</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Yes (physician release)</t>
+          <t>필요(의사)</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="Q19" s="4" t="inlineStr">
         <is>
-          <t>Compose dark-top so white headline reads.</t>
+          <t>상단 다크(화이트 헤드라인).</t>
         </is>
       </c>
     </row>
@@ -2181,27 +2181,27 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 35)</t>
+          <t>스트럭쳐 리셋 LP Hero(35행)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>text only on dark</t>
+          <t>다크·텍스트</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Thermage FLX device with tip and CPT cable visible — sense of premium engineering.</t>
+          <t>써마지 FLX+팁+CPT, 프리미엄 엔지니어링 느낌.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2211,22 +2211,22 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>soft moody premium</t>
+          <t>뮤지엄톤</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Thermage branding subtle, hand entering frame</t>
+          <t>써마지, 손(선택)</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>patient body, used disposables in frame</t>
+          <t>환자 신체, 사용 후 일회품 노출</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="Q20" s="4" t="inlineStr">
         <is>
-          <t>VIP slot LP — emphasize premium feel.</t>
+          <t>프리미엄 VIP 랜딩 톤.</t>
         </is>
       </c>
     </row>
@@ -2268,27 +2268,27 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 35)</t>
+          <t>콜라겐 빌더 LP Hero(35행)</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>text only on dark</t>
+          <t>다크·텍스트</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Tray of skin-booster vials (Rejuran / Juvelook) being arranged by gloved hand — clinical premium.</t>
+          <t>스킨부스터 바이알(리쥬란/쥬베룩) 트레이+장갑(오버헤드).</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -2298,22 +2298,22 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>soft moody premium with single rim light</t>
+          <t>뮤지엄+단일 림</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>vials with manufacturer branding, sterile tray, gloved hand</t>
+          <t>제조사 밍, 멸균 트레이, 장갑</t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>opened needle caps in unsafe orientation, patient</t>
+          <t>부적절한 캡 개방, 환자</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="Q21" s="4" t="inlineStr">
         <is>
-          <t>Shows 'design before injection' tone.</t>
+          <t>‘주입 전 디자인’ 톤.</t>
         </is>
       </c>
     </row>
@@ -2355,27 +2355,27 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 35)</t>
+          <t>볼륨·차마카세 LP Hero(35행)</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>text only on dark</t>
+          <t>다크·텍스트</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Physician holding face-mapping marker over a face-anatomy diagram or 3D mannequin head — design intent.</t>
+          <t>해부도·3D 머리 모형+마커(디자인 의도, 실환자 X).</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2385,22 +2385,22 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>soft moody premium</t>
+          <t>뮤지엄톤</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>anatomy mannequin or printed face map, marker, gloved hand</t>
+          <t>해부/맨네킨, 마커, 장갑</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>photo of real patient, comparing brands</t>
+          <t>실제 환자 사진, 브랜드 비교 연출</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>Yes (physician release)</t>
+          <t>필요(의사)</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="Q22" s="4" t="inlineStr">
         <is>
-          <t>Doubles for 'Designed for Harmony' section.</t>
+          <t>하모니 섹션과 겸용.</t>
         </is>
       </c>
     </row>
@@ -2442,27 +2442,27 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 14)</t>
+          <t>결정보호 LP Hero(14행)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Calm consultation desk with iPad showing planning visual, paper plan, glass of water, no people — invitation to think.</t>
+          <t>iPad(플랜), 종이, 물, 생화 — 인물 없이(사고 유도).</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -2472,22 +2472,22 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>soft daylight, airy minimalist</t>
+          <t>밝은 공기감, 미니멀</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>iPad with placeholder plan visual, printed plan card, fresh stem, branded notebook</t>
+          <t>아이패드(플랜), 노트, 브랜딩</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>phones, names, real patient data</t>
+          <t>개인정보, 전화, 이름</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="Q23" s="4" t="inlineStr">
         <is>
-          <t>Reuse for /metacell-protocol footer CTA and /design-method intro.</t>
+          <t>메타셀 푸터·디자인방식 intro 재사용.</t>
         </is>
       </c>
     </row>
@@ -2529,27 +2529,27 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 37)</t>
+          <t>디자인방식 LP Hero(37행)</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Physician hand drawing facial vector lines on a printed face anatomy sheet — anatomical design feel.</t>
+          <t>해부 시트+페이스 벡터(손만).</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2559,22 +2559,22 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>warm daylight, focused desk lamp</t>
+          <t>따뜻한 데이+책상램프</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>anatomy diagram, fineliner or marker, hand only</t>
+          <t>해부도, 펜, 손</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>patient photo on the desk, brand logos of devices</t>
+          <t>책상의 환자 사진, 기기로고(과도)</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Yes (physician release, hand-only OK)</t>
+          <t>필요(의사, 손만 OK)</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="Q24" s="4" t="inlineStr">
         <is>
-          <t>Captures 'Anatomical Design Workflow' theme.</t>
+          <t>해부·디자인 워크플로우 톤.</t>
         </is>
       </c>
     </row>
@@ -2616,27 +2616,27 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Anatomical Design Workflow steps (line 130)</t>
+          <t>해부적 디자인 6스텝(130행)</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>text only, six step cards</t>
+          <t>텍스트 6칸</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Series of six matched close-ups: assessment notes, planning iPad, vector overlay sheet, structural blueprint, micro-detail tools, depth-safety calibration card.</t>
+          <t>동일 제스: 메모,아이패드,벡터,블루프린트,미세,깊이안전—클로즈6장(정사각).</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>square (1:1)</t>
+          <t>정사각 1:1</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -2646,22 +2646,22 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>warm daylight, consistent across all six</t>
+          <t>데이, 6장 동일</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>consistent surface (same desk), one hand max per frame</t>
+          <t>동일 책상, 화면마다 손 1쌍 이하</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>patient identifiers, mismatched lighting</t>
+          <t>식별자, 조명 불일치</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Yes (physician release for hands)</t>
+          <t>필요(의사 손)</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
@@ -2671,12 +2671,12 @@
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>6 cards (matched set)</t>
+          <t>6장(세트)</t>
         </is>
       </c>
       <c r="Q25" s="4" t="inlineStr">
         <is>
-          <t>Shoot all six in one sitting for visual consistency.</t>
+          <t>한 세션에 연촬.</t>
         </is>
       </c>
     </row>
@@ -2703,27 +2703,27 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 17)</t>
+          <t>압구정(외국인) LP Hero(17행)</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Combination split: building facade left + cropped Apgujeong-rodeo skyline right, OR a single hero of the 5F approach with district context through window.</t>
+          <t>좌:전면 / 우:스카이라인 분할, 또는 5F 창+지구 맥락.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2733,22 +2733,22 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>bright daylight, premium</t>
+          <t>맑고 프리미엄</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>recognizable Apgujeong context + clinic identifier</t>
+          <t>압구정 맥락+클리닉 식별</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>competitor signs</t>
+          <t>경쟁 사인</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="Q26" s="4" t="inlineStr">
         <is>
-          <t>Can compose from existing P0 location shots if shoot day is tight.</t>
+          <t>P0로케이션이 촉박하면 합성.</t>
         </is>
       </c>
     </row>
@@ -2790,27 +2790,27 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 14)</t>
+          <t>시술 FAQ Hero(14행)</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Front-desk concierge at reception with iPad in English UI, calmly answering question (back of patient head visible only).</t>
+          <t>리셥션+아이패드(영문 UI, 환자 뒷통수).</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2820,22 +2820,22 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>warm daylight</t>
+          <t>따뜻한 데이</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>concierge in uniform/blazer, iPad in English UI, branded counter</t>
+          <t>유니폼, 영문, 브랜딩</t>
         </is>
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>real patient face, real iPad data</t>
+          <t>얼굴, 실제 데이터</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Yes (staff release; stand-in patient release)</t>
+          <t>필요(직원+스탠드인)</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="Q27" s="4" t="inlineStr">
         <is>
-          <t>Supports 'English support is real' trust.</t>
+          <t>‘영어 응대 실제’ 신뢰.</t>
         </is>
       </c>
     </row>
@@ -2877,27 +2877,27 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 31)</t>
+          <t>가이드 index Hero(31행)</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Printed Tune Clinic guides / brochures fanned on consultation desk with reading glasses + warm coffee — pre-arrival planning vibe.</t>
+          <t>인쇄 가이드+안경+커피(오버헤드) 입국 전 느낌.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2907,22 +2907,22 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>warm daylight, airy</t>
+          <t>따뜻·에어리</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>branded guide covers (placeholder OK), reading aid, warm cup</t>
+          <t>브랜딩(플레이스홀더 OK)</t>
         </is>
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>competitor brochures in frame</t>
+          <t>다른 병원 브로셔</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="Q28" s="4" t="inlineStr">
         <is>
-          <t>Pair with smaller marquee crop for /guides sub-pages.</t>
+          <t>서브가이드용 마퀴 crop.</t>
         </is>
       </c>
     </row>
@@ -2964,27 +2964,27 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 16) + device cards (line 39)</t>
+          <t>한국 리프팅 가이드 Hero+카드(16·39행)</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Lineup overhead of three lifting devices' branded heads (Ultherapy, Thermage FLX, Oligio/ONDA) on neutral pad — visual encyclopedia.</t>
+          <t>울쎄라·써마·온다(올리지오) 핸드피스 라인(오버헤드) 시각 백과.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2994,22 +2994,22 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral</t>
+          <t>클리니컬</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>three handpieces clearly distinguishable, clean pad</t>
+          <t>3핸드피스, 깨끗한 패드</t>
         </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
         <is>
-          <t>duct tape, dust, mismatched lighting</t>
+          <t>테이프·먼지·불일치 조명</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
@@ -3019,12 +3019,12 @@
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>2 (overhead + 30deg)</t>
+          <t>2(오버+30°)</t>
         </is>
       </c>
       <c r="Q29" s="4" t="inlineStr">
         <is>
-          <t>Each device also gets its own square crop for the four cards.</t>
+          <t>4카드용 정사각 crop 추가.</t>
         </is>
       </c>
     </row>
@@ -3051,27 +3051,27 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 14)</t>
+          <t>울쎄라 vs 써마지 Hero(14행)</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Ultherapy and Thermage FLX devices side by side in same frame, separated by neutral panel — no winner implied.</t>
+          <t>두 기기 동일 프레임+중성 패널(우열 없음).</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -3081,22 +3081,22 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral with soft side fill</t>
+          <t>클리니컬+사이드 필</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>both device fronts, branding subtle but visible</t>
+          <t>전면+밍</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>any visual ranking (e.g. one elevated)</t>
+          <t>한쪽만 도드라지게(우열)</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="Q30" s="4" t="inlineStr">
         <is>
-          <t>Critical to keep visually balanced — equal framing.</t>
+          <t>균형 프레이밍 필수.</t>
         </is>
       </c>
     </row>
@@ -3138,27 +3138,27 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 15) + brand cards (line 36)</t>
+          <t>더말·필러 Hero(15·36행)</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Refrigerated tray of HA filler boxes (Juvederm, Restylane, Belotero, Radiesse) arranged neatly — 'real clinical flow' theme.</t>
+          <t>냉장 트레이+HA(쥬비·레스·벨·라디) 동등 노출(오버헤드).</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -3168,22 +3168,22 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral, slight cool tone</t>
+          <t>클리니컬, 살짝 쿨</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>visible HA filler brand boxes (not expired), gloved hand</t>
+          <t>소비기한 OK 박스, 장갑</t>
         </is>
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>open/used syringes, no brand displayed dominantly larger than others</t>
+          <t>사용된 주사기, 한 브랜드만 강조</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
@@ -3193,12 +3193,12 @@
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>2 (full + tight crop)</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q31" s="4" t="inlineStr">
         <is>
-          <t>Compliance: equal-sized brand presence; do not imply endorsement.</t>
+          <t>브랜드 동등(오해 없이).</t>
         </is>
       </c>
     </row>
@@ -3225,27 +3225,27 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 14) + brand cards (line 35)</t>
+          <t>스킨부스터·재생 Hero(14·35행)</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Tray of skin-booster vials (Rejuran/PDRN, Juvelook, exosomes, Sculptra) with labels visible, neat clinical arrangement.</t>
+          <t>리쥬/PDRN·쥬베·엑소·스컬(라벨) 정돈(오버헤드).</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -3255,22 +3255,22 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral</t>
+          <t>클리니컬</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>four product categories visible, sterile tray</t>
+          <t>4범주, 멸균 트레이</t>
         </is>
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>any brand visually dominant, opened sharps</t>
+          <t>한 브랜드 압도, 열린 샤프</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="Q32" s="4" t="inlineStr">
         <is>
-          <t>Pair with single-product close-ups for the four cards.</t>
+          <t>카드용 단품 클로즈.</t>
         </is>
       </c>
     </row>
@@ -3312,27 +3312,27 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 14)</t>
+          <t>탈모·두피 Hero(14행)</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Scalp-treatment device head over a neutral mannequin scalp model OR overhead of scalp-care vial set + applicator — no real patient.</t>
+          <t>마네킨 두피+기기, 또는 케어 앰플(실환자 X).</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -3342,22 +3342,22 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral</t>
+          <t>클리니컬</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>scalp device or labelled vials, gloved hand</t>
+          <t>기기/바이알, 장갑</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
         <is>
-          <t>visible scalp of real patient, hair loss before/after photos</t>
+          <t>실제 두피, 전후사진</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
@@ -3372,7 +3372,7 @@
       </c>
       <c r="Q33" s="4" t="inlineStr">
         <is>
-          <t>Lower-traffic page; one solid hero is enough.</t>
+          <t>저트래픽, 히어로 1면으로 충분.</t>
         </is>
       </c>
     </row>
@@ -3399,27 +3399,27 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 14) + indication cards (line 30)</t>
+          <t>리프팅 고르는 법 Hero+카드(14·30행)</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Physician's hand drawing four indication zones on printed face diagram (sagging, loose skin, contour collapse, travel timing).</t>
+          <t>4구역(처짐·탄력·윤곽·체류) 해부지+마커(손만).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3429,22 +3429,22 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>warm daylight</t>
+          <t>따뜻한 데이</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>anatomy diagram with annotations, marker</t>
+          <t>해부도+마킹</t>
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr">
         <is>
-          <t>patient photo, brand-name device</t>
+          <t>환자 사진, 기기·브랜드명(과다)</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>Yes (physician release; hand-only OK)</t>
+          <t>필요(의사, 손만)</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
@@ -3459,7 +3459,7 @@
       </c>
       <c r="Q34" s="4" t="inlineStr">
         <is>
-          <t>Same lighting as design-method workflow set.</t>
+          <t>디자인방식과 동일 조명.</t>
         </is>
       </c>
     </row>
@@ -3486,27 +3486,27 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 19)</t>
+          <t>외국인 가이드 Hero(19행)</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Open passport, printed itinerary, branded planning card, AirPods on minimalist desk — 'planning your Seoul trip' overhead.</t>
+          <t>여권(표지만/일반), 일정, 명함, 에어팟(오버헤드) 서울·계획 느낌.</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3516,22 +3516,22 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>warm daylight, airy</t>
+          <t>따뜻·에어리</t>
         </is>
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>passport (cover only or generic), itinerary print, branded card</t>
+          <t>여권(민감X), 일정, 명함</t>
         </is>
       </c>
       <c r="M35" s="4" t="inlineStr">
         <is>
-          <t>real passport photo page, real flight numbers/names</t>
+          <t>사진·페이지, 편명·실명</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="Q35" s="4" t="inlineStr">
         <is>
-          <t>Pair with concierge image for FAQ page.</t>
+          <t>FAQ용 컨시어지와 페어.</t>
         </is>
       </c>
     </row>
@@ -3573,27 +3573,27 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 111)</t>
+          <t>메뉴(가격) Hero(111행)</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>text only on dark</t>
+          <t>다크·텍스트</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Printed Chamaka-se menu booklet on premium paper, edge-lit on stone counter, single fresh stem.</t>
+          <t>차마카세 인쇄 메뉴+스톤+꽃(오버헤드) 스프레드시트 느낌 완화.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3603,22 +3603,22 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>soft moody premium</t>
+          <t>뮤지엄</t>
         </is>
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Tune Clinic-branded menu (placeholder OK), stone surface</t>
+          <t>브랜딩(플레이스홀더 OK), 스톤</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>competitor pricing in shot</t>
+          <t>타 클리닉 가격</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="Q36" s="4" t="inlineStr">
         <is>
-          <t>Helps the price-list page feel less like a spreadsheet.</t>
+          <t>가독+프리미엄.</t>
         </is>
       </c>
     </row>
@@ -3650,7 +3650,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>(equipment library)</t>
+          <t>(장비·라이브러리)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -3660,27 +3660,27 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Ultherapy device close-up</t>
+          <t>장비(라이브러리) — 울쎄라</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Ultherapy device handpiece with Tune branding sticker subtle, mounted on machine.</t>
+          <t>핸드피스+기기, 은은한 튠 스티커, 시리얼 가림.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>square (1:1)</t>
+          <t>정사각 1:1</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3690,22 +3690,22 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral</t>
+          <t>클리니컬</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>Ultherapy branding, serial number obscured</t>
+          <t>울쎄라 밍</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>dust, used gel residue</t>
+          <t>먼지, 잔·젤</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>3 angles</t>
+          <t>각도 3</t>
         </is>
       </c>
       <c r="Q37" s="4" t="inlineStr">
         <is>
-          <t>Reused on signature-lifting, structural-reset, korean-lifting-guide, ultherapy-vs-thermage.</t>
+          <t>시그·스트럭·가이드·vs 다용.</t>
         </is>
       </c>
     </row>
@@ -3737,7 +3737,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>(equipment library)</t>
+          <t>(장비·라이브러리)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -3747,27 +3747,27 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Thermage FLX device close-up</t>
+          <t>장비(라이브러리) — 써마지 FLX</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Thermage FLX tip with CPT cartridge attached, on machine; clean.</t>
+          <t>CPT+팁, 기기(깨끗).</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>square (1:1)</t>
+          <t>정사각 1:1</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3777,22 +3777,22 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral</t>
+          <t>클리니컬</t>
         </is>
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Thermage branding subtle, tip facing camera</t>
+          <t>써마지, 팁 정면</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>dust, used cartridges visible</t>
+          <t>사용 칼트, 먼지</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
@@ -3802,12 +3802,12 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>3 angles</t>
+          <t>각도 3</t>
         </is>
       </c>
       <c r="Q38" s="4" t="inlineStr">
         <is>
-          <t>Reused on structural-reset, ultherapy-vs-thermage.</t>
+          <t>스트럭·vs 다용.</t>
         </is>
       </c>
     </row>
@@ -3824,7 +3824,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>(equipment library)</t>
+          <t>(장비·라이브러리)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -3834,27 +3834,27 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>ONDA Lifting device close-up</t>
+          <t>장비(라이브러리) — 온다 리프팅</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>ONDA microwave-lifting handpiece on machine — distinctive shape.</t>
+          <t>마이크로웨이브·온다 핸드피스(형태 특징).</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>square (1:1)</t>
+          <t>정사각 1:1</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3864,22 +3864,22 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral</t>
+          <t>클리니컬</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>ONDA branding, clean handpiece</t>
+          <t>온다, 깨끗</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>cluttered backdrop</t>
+          <t>뒤 산란(혼잡)</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="Q39" s="4" t="inlineStr">
         <is>
-          <t>Reused on korean-lifting-guide, signature-lifting.</t>
+          <t>한국·시그.</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>(equipment library)</t>
+          <t>(장비·라이브러리)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -3921,27 +3921,27 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>PBM (photobiomodulation) device</t>
+          <t>장비(라이브러리) — PBM(광생체조절)</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>PBM device head with red light visible at low intensity, on stand — minimalist.</t>
+          <t>PBM 헤드+저광 red glow, 환자 없음(미니멀).</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>square (1:1)</t>
+          <t>정사각 1:1</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -3951,22 +3951,22 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>clinical bright neutral with red device glow</t>
+          <t>클리니컬+red glow</t>
         </is>
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>device head, soft red glow, no patient</t>
+          <t>헤드, 은은한 빨강(과노X)</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>overexposed light source</t>
+          <t>광원 과다노출</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="Q40" s="4" t="inlineStr">
         <is>
-          <t>Critical for /metacell-protocol cards.</t>
+          <t>메타셀 카드 핵심.</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>(equipment library)</t>
+          <t>(장비·라이브러리)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -4008,27 +4008,27 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Juvelook syringe / Rejuran vials</t>
+          <t>장비(라이브러리) — 쥬베·리쥬란</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Single Juvelook syringe and Rejuran box arranged with sterile pad — premium product still life.</t>
+          <t>쥬베 針+리쥬 박스+멸균 매트(스틸).</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>square (1:1)</t>
+          <t>정사각 1:1</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -4038,22 +4038,22 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>soft daylight, clean white surface</t>
+          <t>밝은 화이트</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>manufacturer branding intact, lot label obscured</t>
+          <t>밍, 로트(가리기)</t>
         </is>
       </c>
       <c r="M41" s="4" t="inlineStr">
         <is>
-          <t>opened needle, expired packaging</t>
+          <t>캡이 열린 바늘(샤프), 유통기한 지난</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
@@ -4063,12 +4063,12 @@
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>3 (separate + together)</t>
+          <t>3(분리+합)</t>
         </is>
       </c>
       <c r="Q41" s="4" t="inlineStr">
         <is>
-          <t>Reused on collagen-builder, skin-boosters, blog hero pool.</t>
+          <t>콜라겐·스킨·블로그.</t>
         </is>
       </c>
     </row>
@@ -4095,27 +4095,27 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>IV sedation chair</t>
+          <t>IV(정맥) 진정(메뉴/스트럭쳐)</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Empty IV-sedation recliner with warm blanket folded, side table with water — calm comfort.</t>
+          <t>빈 IV 리클라이너+담요+물(환자 없이).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -4125,22 +4125,22 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>warm daylight + warm tungsten</t>
+          <t>데이+웜 텅</t>
         </is>
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>recliner, folded throw, side table, no patient</t>
+          <t>리클라·담요·협탁</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>visible used IV bags, monitors with data</t>
+          <t>시술·모니터 개인정보</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O42" s="2" t="inlineStr">
@@ -4155,7 +4155,7 @@
       </c>
       <c r="Q42" s="4" t="inlineStr">
         <is>
-          <t>High emotional payoff for premium audiences.</t>
+          <t>프리미엄 감성.</t>
         </is>
       </c>
     </row>
@@ -4182,27 +4182,27 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Recovery lounge</t>
+          <t>리커버리 라운지(메뉴/스트럭쳐)</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Recovery lounge wide — ambient lighting, soft seating, fresh tea station, quiet plant — no patient.</t>
+          <t>라운지 와이드, 티, 식물(환자 없이).</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -4212,22 +4212,22 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>warm tungsten, soothing premium</t>
+          <t>웜 티(진정·프리미엄)</t>
         </is>
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>ambient seating, tea station, plants</t>
+          <t>착석, 티, 식물</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>patients, used towels</t>
+          <t>환자, 사용 타올(과다)</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O43" s="2" t="inlineStr">
@@ -4237,12 +4237,12 @@
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>3 angles</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q43" s="4" t="inlineStr">
         <is>
-          <t>Shoot pre-opening for empty space.</t>
+          <t>오픈 전 공실.</t>
         </is>
       </c>
     </row>
@@ -4259,7 +4259,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -4269,27 +4269,27 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Treatment room wide</t>
+          <t>시술실(전역 재사용)</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Empty treatment room with reclined bed, device draped, accent lamp — 'private and clean' tone.</t>
+          <t>빈 시술베드+덮인 기기+램프 — 프라이빗·클린.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -4299,22 +4299,22 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>warm clinical neutral</t>
+          <t>웜 클리니컬</t>
         </is>
       </c>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>treatment bed, draped device, branded touches</t>
+          <t>베드, 드레이프, 터치</t>
         </is>
       </c>
       <c r="M44" s="4" t="inlineStr">
         <is>
-          <t>biohazard bins prominent, used disposables</t>
+          <t>이물함·사용 1회품(과다)</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
@@ -4324,12 +4324,12 @@
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>3 (different rooms)</t>
+          <t>3(실 3곳)</t>
         </is>
       </c>
       <c r="Q44" s="4" t="inlineStr">
         <is>
-          <t>Reusable across procedure LPs.</t>
+          <t>LP 다용.</t>
         </is>
       </c>
     </row>
@@ -4346,7 +4346,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -4356,27 +4356,27 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>Consultation room wide</t>
+          <t>상담실(전역)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Consultation room wide — desk with iPad, two chairs, warm lamp, anatomy print framed on wall.</t>
+          <t>데스크·아이패드·2의자·램프·해부액자.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -4386,22 +4386,22 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>warm daylight + tungsten lamp</t>
+          <t>데이+램프</t>
         </is>
       </c>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>desk, two chairs, anatomy/aesthetic art</t>
+          <t>2의자, 액자</t>
         </is>
       </c>
       <c r="M45" s="4" t="inlineStr">
         <is>
-          <t>patient charts visible, prices on screen</t>
+          <t>차트·가격</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
@@ -4416,7 +4416,7 @@
       </c>
       <c r="Q45" s="4" t="inlineStr">
         <is>
-          <t>Reused on /booking, /design-method, /decision-protection.</t>
+          <t>예약·디자인·결정.</t>
         </is>
       </c>
     </row>
@@ -4443,27 +4443,27 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Hero (line 55)</t>
+          <t>갤러리 Hero(55행) — ‘크롬’(전후 X)</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>text only on dark</t>
+          <t>다크·텍스트</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>Process imagery — physician's hand placing a printed plan card next to closed before/after photo envelopes — implies documentation without revealing patients.</t>
+          <t>플랜카드+봉투(전후 X, 문서 느낌만).</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4473,22 +4473,22 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>soft moody premium</t>
+          <t>뮤지엄</t>
         </is>
       </c>
       <c r="L46" s="4" t="inlineStr">
         <is>
-          <t>plan card, archive folder/envelope, gloved hand</t>
+          <t>케이스, 폴더, 장갑</t>
         </is>
       </c>
       <c r="M46" s="4" t="inlineStr">
         <is>
-          <t>any actual before/after image (separate consent track)</t>
+          <t>실제 전·후 이미지(별도 동의)</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="Q46" s="4" t="inlineStr">
         <is>
-          <t>Real before/after photos require their own patient release process — this row covers chrome only.</t>
+          <t>실전·후는 별도 릴리즈 트랙.</t>
         </is>
       </c>
     </row>
@@ -4530,27 +4530,27 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Page header</t>
+          <t>예약 관리(헤더)</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>text only / form chrome</t>
+          <t>폼/텍스트</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>Calendar and pen on neutral surface — manage-your-booking visual cue.</t>
+          <t>달력+펜(중립면) — 관리·변경 느낌.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -4560,22 +4560,22 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>soft daylight</t>
+          <t>소프트 데이</t>
         </is>
       </c>
       <c r="L47" s="4" t="inlineStr">
         <is>
-          <t>undated calendar, pen, branded card</t>
+          <t>날짜 X 달력, 펜, 명함</t>
         </is>
       </c>
       <c r="M47" s="4" t="inlineStr">
         <is>
-          <t>real patient name on calendar</t>
+          <t>실명, 예약</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr">
@@ -4590,7 +4590,7 @@
       </c>
       <c r="Q47" s="4" t="inlineStr">
         <is>
-          <t>Optional — useful if we later add a header strip image.</t>
+          <t>스트립 이미지—선택.</t>
         </is>
       </c>
     </row>
@@ -4617,27 +4617,27 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Hero</t>
+          <t>빠른문의(컨설트) Hero</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>Physician at desk with phone in hand mid-call (back to camera) — 'we'll get back to you' reassurance.</t>
+          <t>데스크·전화(뒤통수) — ‘다시 연락’ 안심.”</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -4647,22 +4647,22 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>warm daylight</t>
+          <t>따뜻·데이</t>
         </is>
       </c>
       <c r="L48" s="4" t="inlineStr">
         <is>
-          <t>white-coat back, branded notepad, calm desk</t>
+          <t>가운만 보이는 뒷모습(가능), 노트, 차분</t>
         </is>
       </c>
       <c r="M48" s="4" t="inlineStr">
         <is>
-          <t>visible phone screen with names</t>
+          <t>이름·화면</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>Yes (staff release)</t>
+          <t>필요(직원)</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr">
@@ -4677,7 +4677,7 @@
       </c>
       <c r="Q48" s="4" t="inlineStr">
         <is>
-          <t>Lower priority — current consult flow is mostly form.</t>
+          <t>낮은 우선. 주로 폼.</t>
         </is>
       </c>
     </row>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>(blog)</t>
+          <t>(블로그)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -4704,27 +4704,27 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Blog hero generic pool</t>
+          <t>블로그(EN) — 범용 히어로 풀 3</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>Three reusable detail crops: (a) anatomy print + marker, (b) printed Tune brochure on stone, (c) macro of fresh florals at reception. To be assigned to blog posts based on topic.</t>
+          <t>①해부+마커 ②튠 팜프 ③리셥션·꽃(맥락별로 배정).</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>close-up</t>
+          <t>클로즈업/와이드</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -4734,22 +4734,22 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>warm daylight</t>
+          <t>따뜻·데이</t>
         </is>
       </c>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>brand-consistent detail, no patient</t>
+          <t>일관·브랜딩, 환자X</t>
         </is>
       </c>
       <c r="M49" s="4" t="inlineStr">
         <is>
-          <t>topic-specific elements (kept generic)</t>
+          <t>주제만 너무 구체(범용 유지)</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O49" s="2" t="inlineStr">
@@ -4759,12 +4759,12 @@
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>3 generic crops</t>
+          <t>3장(범용)</t>
         </is>
       </c>
       <c r="Q49" s="4" t="inlineStr">
         <is>
-          <t>Editor maps each blog post to one of the 3 crops; topic-specific posts can be upgraded later.</t>
+          <t>에디터·포스트에 매핑, 후일 업그레이드 가능.</t>
         </is>
       </c>
     </row>
@@ -4781,7 +4781,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>(global footer)</t>
+          <t>(푸터·전역)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -4791,27 +4791,27 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Footer / contact strip</t>
+          <t>푸터/연락(황혼·외관)</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>Wide of building exterior at dusk with warm interior glow — quiet brand close.</t>
+          <t>일몰+창빛·건물(조용한 엔딩).</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>wide</t>
+          <t>와이드</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>landscape (16:9)</t>
+          <t>가로 16:9</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -4821,22 +4821,22 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>dusk premium, warm window glow</t>
+          <t>황혼+웜</t>
         </is>
       </c>
       <c r="L50" s="4" t="inlineStr">
         <is>
-          <t>building, lit windows, sense of closure</t>
+          <t>건물·빛</t>
         </is>
       </c>
       <c r="M50" s="4" t="inlineStr">
         <is>
-          <t>people in frame, headlights blowing exposure</t>
+          <t>인물, 헤드라이트 과다</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O50" s="2" t="inlineStr">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="Q50" s="4" t="inlineStr">
         <is>
-          <t>Captures end-of-day brand mood.</t>
+          <t>보너스. ~18:00·재방문.</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4868,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -4878,27 +4878,27 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Concierge candid (English-speaking)</t>
+          <t>컨시어지(영어) 캔디드</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>English-speaking concierge laughing with stand-in international patient — natural candid energy.</t>
+          <t>영어·스탠드인(자연) 웃음 톤.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -4908,22 +4908,22 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>warm daylight</t>
+          <t>따뜻</t>
         </is>
       </c>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>concierge in uniform, English signage subtle</t>
+          <t>유니폼, 은은한 영문</t>
         </is>
       </c>
       <c r="M51" s="4" t="inlineStr">
         <is>
-          <t>forced smile, stiff pose</t>
+          <t>과한 포즈</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>Yes (staff + stand-in release)</t>
+          <t>필요(직원+스탠드인)</t>
         </is>
       </c>
       <c r="O51" s="2" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="Q51" s="4" t="inlineStr">
         <is>
-          <t>Use sparingly; great for FAQ + international guide.</t>
+          <t>FAQ·가이드. 과다사용X.</t>
         </is>
       </c>
     </row>
@@ -4955,7 +4955,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -4965,27 +4965,27 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Skincare / aftercare product line</t>
+          <t>스킨케어(애프터) 세트</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>Aftercare product set on counter — sun protection, calming serum, sheet mask.</t>
+          <t>선·세럼·시트(애프터).</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>overhead</t>
+          <t>탑뷰</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>square (1:1)</t>
+          <t>정사각 1:1</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -4995,22 +4995,22 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>soft daylight</t>
+          <t>데이</t>
         </is>
       </c>
       <c r="L52" s="4" t="inlineStr">
         <is>
-          <t>aftercare set, branded card</t>
+          <t>애프터+명함</t>
         </is>
       </c>
       <c r="M52" s="4" t="inlineStr">
         <is>
-          <t>competitor brands without permission</t>
+          <t>무허가 타사</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O52" s="2" t="inlineStr">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="Q52" s="4" t="inlineStr">
         <is>
-          <t>Useful for blog hero pool and recovery posts.</t>
+          <t>블로그·휴지용.</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5042,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -5052,27 +5052,27 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>View from clinic window</t>
+          <t>5층 창(전역) — 감성</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>text only</t>
+          <t>텍스트만</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>View through 5F window of Apgujeong street — soft focus on indoor plant in foreground.</t>
+          <t>창+거리(전경) 전경=식물(소프트).</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>미디엄</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>landscape (3:2)</t>
+          <t>가로 3:2</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
@@ -5082,22 +5082,22 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>bright daylight + indoor warm</t>
+          <t>데이+실내</t>
         </is>
       </c>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>window framing, district view, plant detail</t>
+          <t>창, 지구, 식물</t>
         </is>
       </c>
       <c r="M53" s="4" t="inlineStr">
         <is>
-          <t>patient at window, identifiable signage outside</t>
+          <t>창에 환자, 외부 식별 간판(과다)</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="O53" s="2" t="inlineStr">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="Q53" s="4" t="inlineStr">
         <is>
-          <t>Atmospheric; reuses across blog and global imagery.</t>
+          <t>분위기·재사용·블로그.</t>
         </is>
       </c>
     </row>
@@ -5143,12 +5143,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>page</t>
+          <t>페이지(URL/범주)</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>page_file</t>
+          <t>소스 파일</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -5168,12 +5168,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>합계</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>shoot_day_notes</t>
+          <t>촬영·편집 메모</t>
         </is>
       </c>
     </row>
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Home - highest reuse. Pair Block A exterior + Block E portraits to land 5/6 ad launch.</t>
+          <t>메인 — 재촬·재활용 최다. A(외부)+E(의료진)로 5/6 광고 런칭 핵심을 커버.</t>
         </is>
       </c>
     </row>
@@ -5231,7 +5231,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Pair with Dr. Cha environmental from Block E; one overhead desk shot covers hero + success.</t>
+          <t>E의 상담·환경과 맞출 것. 히어로+완료: 탑뷰 데스크 1장이면 둘 다 대응 가능.</t>
         </is>
       </c>
     </row>
@@ -5260,14 +5260,14 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Flagship LP - block off Dr. Cha or Dr. Ju gloved hands at start of Block D for the 3 build crops.</t>
+          <t>핵심 LP. D시작 직전 차/주+장갑, 3빌드(울/써/PBM)는 같은 조명으로 연촬.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -5289,14 +5289,14 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Reused across many pages - shoot once, wire everywhere.</t>
+          <t>한 번 촬영해 사이트 여러 섹션에 연결(개발팀이 배치).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -5318,14 +5318,14 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Reused across many pages - shoot once, wire everywhere.</t>
+          <t>한 번 촬영해 사이트 여러 섹션에 연결(개발팀이 배치).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -5347,7 +5347,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Reused across many pages - shoot once, wire everywhere.</t>
+          <t>한 번 촬영해 사이트 여러 섹션에 연결(개발팀이 배치).</t>
         </is>
       </c>
     </row>
@@ -5779,7 +5779,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>(equipment library)</t>
+          <t>(장비·라이브러리)</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -5801,7 +5801,7 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Coordinate with nurse during Block D to ensure devices are not in patient use.</t>
+          <t>D·D-2 — 간호와 협의, 환자 시술과 시간 겹침 방지.</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>(global)</t>
+          <t>(전역)</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -5880,7 +5880,7 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Reused across many pages - shoot once, wire everywhere.</t>
+          <t>한 번 촬영해 사이트 여러 섹션에 연결(개발팀이 배치).</t>
         </is>
       </c>
     </row>
@@ -5962,7 +5962,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>(blog)</t>
+          <t>(블로그)</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -5984,14 +5984,14 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>P2 - generic crops only; don't slow other blocks for these.</t>
+          <t>P2(우선순위 낮음) — 앞 구간에 지면 금지.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>(global footer)</t>
+          <t>(푸터·전역)</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -6013,14 +6013,14 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Revisit at dusk (18:00) for the warm-glow exterior variant.</t>
+          <t>18:00 전후 ‘황혼+창빛’ 외부 1장(옵션이지만 톤 좋음).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>합계</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr"/>
@@ -6063,44 +6063,44 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>block</t>
+          <t>구간</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>time_window</t>
+          <t>시간대</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>duration_min</t>
+          <t>소요(분)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>kit_lighting</t>
+          <t>조명·장비</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>covered_row_ids</t>
+          <t>포함 행 ID</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>row_count</t>
+          <t>행 수</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Block A - Exterior + district context</t>
+          <t>A구간 — 외부 전경 + 압구정 맥락</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>09:30 - 11:00 (morning daylight)</t>
+          <t>09:30–11:00 (아침 자연광)</t>
         </is>
       </c>
       <c r="C2" s="4" t="n">
@@ -6108,8 +6108,8 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Lighting: Natural daylight, no flash; consider polarizer for storefront glass
-Kit: 24-70mm, 16-35mm wide, polarizer, ND8, no tripod (handheld OK at this hour)</t>
+          <t>조명: 자연광, 섬광 비권장, 유리면은 편광 필터(선택).
+장비: 24–70mm, 16–35mm(와이드), 편광, ND8, 삼각대 생략 가능(핸드헬드).</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -6124,12 +6124,12 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Block B - 5F approach + reception + waiting</t>
+          <t>B구간 — 5층 동선 + 리셉션 + 대기</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>11:00 - 12:30 (pre-opening for empty rooms)</t>
+          <t>11:00–12:30 (오픈 전 공실 권장)</t>
         </is>
       </c>
       <c r="C3" s="4" t="n">
@@ -6137,8 +6137,8 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Lighting: Mixed daylight + warm tungsten; bring small bounce + softbox
-Kit: 24-70mm, 35mm prime, tripod, 1 softbox, white bounce</t>
+          <t>조명: 자연광+웜 텅, 소형 바운스·소프트박스.
+장비: 24–70mm, 35mm 프라임, 삼각대, 소프트박스1, 흰 반사.</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -6153,12 +6153,12 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Block C - Consultation rooms + treatment rooms</t>
+          <t>C구간 — 상담실 + 시술실 + 문서/플랜 연출</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>13:00 - 15:00 (skip lunch hour overlap with patients)</t>
+          <t>13:00–15:00 (점심·환자 인수인계 피할 것)</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
@@ -6166,8 +6166,8 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Lighting: Daylight + tungsten; ensure no patient handover during shoot
-Kit: Tripod for overhead rig, 35mm/50mm primes, color checker, mannequin head if available</t>
+          <t>조명: 데이+텅, 촬영 시 환자·동선 충돌 없게.
+장비: 탑뷨용 리그·삼각대, 35/50mm, 컬러체커, 마네킨(가능 시).</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -6182,12 +6182,12 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Block D - Equipment close-ups</t>
+          <t>D구간 — 장비 클로즈업(울/써/스킨부스터·필·두피 등)</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>15:00 - 16:30 (between booked slots; coordinate with nurse)</t>
+          <t>15:00–16:30 (시술 슬롯 틈, 간호와 협의)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
@@ -6195,8 +6195,8 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Lighting: Clean clinical neutral; one warm rim light
-Kit: Macro 100mm, 50mm, tripod, two softboxes, gel filters, sterile pad set, color checker</t>
+          <t>조명: 클리니컬 중성 + 웜 림 1.
+장비: 매크로 100mm, 50mm, 삼각대, 소프트2, 젤, 멸균매트, 컬러체커.</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -6211,12 +6211,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Block D-2 - PBM + product still lifes</t>
+          <t>D-2구간 — PBM + 쥬베/리쥬 스틸</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>16:30 - 17:15</t>
+          <t>16:30–17:15</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
@@ -6224,8 +6224,8 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Lighting: Same setup as Block D
-Kit: (continuation of Block D)</t>
+          <t>조명: D구간과 동일 셋업.
+장비: D구간 연장(같은 조명).</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -6240,12 +6240,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Block E - Physician portraits</t>
+          <t>E구간 — 의료진 포트(차·주)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>17:30 - 19:00 (after patient hours; quiet space)</t>
+          <t>17:30–19:00 (진료·환자 희소 시간대)</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
@@ -6253,8 +6253,8 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Lighting: Window daylight + reflector; backup softbox if cloudy
-Kit: 85mm portrait prime, 50mm, large reflector, softbox, lapel/clip mics if also recording video B-roll</t>
+          <t>조명: 창가 자연광+반사판, 흐리면 소프트박스 백업.
+장비: 85mm(인물), 50mm, 대형 반사, 소프트, B롤·영상 시 라벨/클립 마이크.</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -6269,12 +6269,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Block F - Comfort + amenity (post-hours)</t>
+          <t>F구간 — IV·라운지(퇴근 후)</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>19:00 - 19:45 (lights warm, lounge calm)</t>
+          <t>19:00–19:45 (웜조명, 라운지 캄)</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
@@ -6282,8 +6282,8 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Lighting: Warm tungsten + soft fill
-Kit: 24-70mm, tripod, 1 softbox</t>
+          <t>조명: 웜 텅+소프트 필.
+장비: 24–70mm, 삼각대, 소프트1.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -6298,12 +6298,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Block G - Generic blog hero pool + leftover details</t>
+          <t>G구간 — 블로그 범용 + 잔여 컷(백스톱)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Backstop slot — flex into other blocks if time allows</t>
+          <t>다른 구간·여유에 따라 탄력 운용</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
@@ -6311,8 +6311,8 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Lighting: As needed
-Kit: (uses leftover setups)</t>
+          <t>조명: 씬에 맞게.
+장비: 앞선 셋업 재활용.</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -6327,7 +6327,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Total scheduled minutes</t>
+          <t>총 예정 시간(분, 장비·이동은 별도)</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr"/>

</xml_diff>